<commit_message>
Update delete bon opp
</commit_message>
<xml_diff>
--- a/playwright-test-report.xlsx
+++ b/playwright-test-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
   <si>
     <t>FORM TEST CASE AUTOMATION</t>
   </si>
@@ -25,7 +25,7 @@
     <t>MENU :</t>
   </si>
   <si>
-    <t>BONOPP</t>
+    <t>ABOUT</t>
   </si>
   <si>
     <t>VERSI :</t>
@@ -37,7 +37,7 @@
     <t>TANGGAL :</t>
   </si>
   <si>
-    <t>10/3/2026</t>
+    <t>11/3/2026</t>
   </si>
   <si>
     <t>NO</t>
@@ -70,25 +70,67 @@
     <t>File Spec</t>
   </si>
   <si>
-    <t>TC_D_001</t>
+    <t>TC_A_001</t>
   </si>
   <si>
     <t>Chromium</t>
   </si>
   <si>
+    <t>POSITIVE</t>
+  </si>
+  <si>
+    <t>Click About</t>
+  </si>
+  <si>
+    <t>passed</t>
+  </si>
+  <si>
+    <t>Ali Bunyamin</t>
+  </si>
+  <si>
+    <t>C:\Automation Apps\playwright with codegen\test\About-positive.spec.js</t>
+  </si>
+  <si>
+    <t>TC_C_001</t>
+  </si>
+  <si>
+    <t>CHECKOUT</t>
+  </si>
+  <si>
+    <t>Add To Cart &amp; Checkout Product</t>
+  </si>
+  <si>
+    <t>C:\Automation Apps\playwright with codegen\test\Checkout-positive.spec.js</t>
+  </si>
+  <si>
+    <t>TC_L_001</t>
+  </si>
+  <si>
+    <t>LOGIN</t>
+  </si>
+  <si>
+    <t>Login Positif</t>
+  </si>
+  <si>
+    <t>C:\Automation Apps\playwright with codegen\test\Login-positive.spec.js</t>
+  </si>
+  <si>
+    <t>TC_L_002</t>
+  </si>
+  <si>
     <t>GENERAL</t>
   </si>
   <si>
-    <t>Delete Bon</t>
-  </si>
-  <si>
-    <t>passed</t>
-  </si>
-  <si>
-    <t>Ali Bunyamin</t>
-  </si>
-  <si>
-    <t>C:\Automation Apps\playwright with codegen\test\BonOpp.spec.js</t>
+    <t>Login Negatif (username invalid)</t>
+  </si>
+  <si>
+    <t>C:\Automation Apps\playwright with codegen\test\Login-negatif.spec.js</t>
+  </si>
+  <si>
+    <t>TC_L_003</t>
+  </si>
+  <si>
+    <t>Login Negatif (password invalid)</t>
   </si>
 </sst>
 </file>
@@ -488,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:J9"/>
+  <dimension ref="A2:J13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -599,13 +641,141 @@
         <v>23</v>
       </c>
       <c r="H9">
-        <v>7093</v>
+        <v>7178</v>
       </c>
       <c r="I9" t="s">
         <v>24</v>
       </c>
       <c r="J9" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H10">
+        <v>7706</v>
+      </c>
+      <c r="I10" t="s">
+        <v>24</v>
+      </c>
+      <c r="J10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11">
+        <v>1011</v>
+      </c>
+      <c r="I11" t="s">
+        <v>24</v>
+      </c>
+      <c r="J11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H12">
+        <v>2264</v>
+      </c>
+      <c r="I12" t="s">
+        <v>24</v>
+      </c>
+      <c r="J12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H13">
+        <v>935</v>
+      </c>
+      <c r="I13" t="s">
+        <v>24</v>
+      </c>
+      <c r="J13" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix report excel & add test
</commit_message>
<xml_diff>
--- a/playwright-test-report.xlsx
+++ b/playwright-test-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="51">
   <si>
     <t>FORM TEST CASE AUTOMATION</t>
   </si>
@@ -19,118 +19,151 @@
     <t>PROGRAM :</t>
   </si>
   <si>
-    <t>PRODUKSI</t>
+    <t>saucedemo.com</t>
   </si>
   <si>
     <t>MENU :</t>
   </si>
   <si>
+    <t>CHECKOUT</t>
+  </si>
+  <si>
+    <t>VERSI :</t>
+  </si>
+  <si>
+    <t>DEFAULT</t>
+  </si>
+  <si>
+    <t>TANGGAL :</t>
+  </si>
+  <si>
+    <t>11/3/2026</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>PLATFORM/BROWSER</t>
+  </si>
+  <si>
+    <t>PRE-REQUIREMENT</t>
+  </si>
+  <si>
+    <t>KIND OF TEST</t>
+  </si>
+  <si>
+    <t>DESCRIPTION</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>Duration (ms)</t>
+  </si>
+  <si>
+    <t>EXECUTED BY</t>
+  </si>
+  <si>
+    <t>File Spec</t>
+  </si>
+  <si>
+    <t>TC_C_001</t>
+  </si>
+  <si>
+    <t>chromium</t>
+  </si>
+  <si>
+    <t>POSITIVE</t>
+  </si>
+  <si>
+    <t>Add To Cart &amp; Checkout Product</t>
+  </si>
+  <si>
+    <t>passed</t>
+  </si>
+  <si>
+    <t>Ali Bunyamin</t>
+  </si>
+  <si>
+    <t>C:\Automation Apps\playwright with codegen\test\Checkout-positive.spec.js</t>
+  </si>
+  <si>
+    <t>TC_A_001</t>
+  </si>
+  <si>
     <t>ABOUT</t>
   </si>
   <si>
-    <t>VERSI :</t>
-  </si>
-  <si>
-    <t>DEFAULT</t>
-  </si>
-  <si>
-    <t>TANGGAL :</t>
-  </si>
-  <si>
-    <t>11/3/2026</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>PLATFORM/BROWSER</t>
-  </si>
-  <si>
-    <t>PRE-REQUIREMENT</t>
-  </si>
-  <si>
-    <t>KIND OF TEST</t>
-  </si>
-  <si>
-    <t>DESCRIPTION</t>
-  </si>
-  <si>
-    <t>STATUS</t>
-  </si>
-  <si>
-    <t>Duration (ms)</t>
-  </si>
-  <si>
-    <t>EXECUTED BY</t>
-  </si>
-  <si>
-    <t>File Spec</t>
-  </si>
-  <si>
-    <t>TC_A_001</t>
-  </si>
-  <si>
-    <t>Chromium</t>
-  </si>
-  <si>
-    <t>POSITIVE</t>
-  </si>
-  <si>
     <t>Click About</t>
   </si>
   <si>
-    <t>passed</t>
-  </si>
-  <si>
-    <t>Ali Bunyamin</t>
-  </si>
-  <si>
     <t>C:\Automation Apps\playwright with codegen\test\About-positive.spec.js</t>
   </si>
   <si>
-    <t>TC_C_001</t>
-  </si>
-  <si>
-    <t>CHECKOUT</t>
-  </si>
-  <si>
-    <t>Add To Cart &amp; Checkout Product</t>
-  </si>
-  <si>
-    <t>C:\Automation Apps\playwright with codegen\test\Checkout-positive.spec.js</t>
+    <t>TC_L_002</t>
+  </si>
+  <si>
+    <t>LOGIN</t>
+  </si>
+  <si>
+    <t>NEGATIVE</t>
+  </si>
+  <si>
+    <t>Login (username invalid)</t>
+  </si>
+  <si>
+    <t>C:\Automation Apps\playwright with codegen\test\Login-negative.spec.js</t>
   </si>
   <si>
     <t>TC_L_001</t>
   </si>
   <si>
-    <t>LOGIN</t>
-  </si>
-  <si>
     <t>Login Positif</t>
   </si>
   <si>
     <t>C:\Automation Apps\playwright with codegen\test\Login-positive.spec.js</t>
   </si>
   <si>
-    <t>TC_L_002</t>
-  </si>
-  <si>
-    <t>GENERAL</t>
-  </si>
-  <si>
-    <t>Login Negatif (username invalid)</t>
-  </si>
-  <si>
-    <t>C:\Automation Apps\playwright with codegen\test\Login-negatif.spec.js</t>
-  </si>
-  <si>
     <t>TC_L_003</t>
   </si>
   <si>
-    <t>Login Negatif (password invalid)</t>
+    <t>Login (password invalid)</t>
+  </si>
+  <si>
+    <t>Login (username password invalid)</t>
+  </si>
+  <si>
+    <t>LOGOUT</t>
+  </si>
+  <si>
+    <t>C:\Automation Apps\playwright with codegen\test\Logout-positive.spec.js</t>
+  </si>
+  <si>
+    <t>TC_P_001</t>
+  </si>
+  <si>
+    <t>PRODUCT</t>
+  </si>
+  <si>
+    <t>Look for detail product</t>
+  </si>
+  <si>
+    <t>C:\Automation Apps\playwright with codegen\test\Product-positive.spec.js</t>
+  </si>
+  <si>
+    <t>TC_P_002</t>
+  </si>
+  <si>
+    <t>Sort by product</t>
+  </si>
+  <si>
+    <t>firefox</t>
+  </si>
+  <si>
+    <t>webkit</t>
   </si>
 </sst>
 </file>
@@ -172,7 +205,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -180,17 +213,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin">
+        <color rgb="FFE0E0E0"/>
+      </top>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -530,7 +573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:J13"/>
+  <dimension ref="A2:J35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -619,163 +662,867 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="A9" s="3">
         <v>1</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="E9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H9">
-        <v>7178</v>
-      </c>
-      <c r="I9" t="s">
-        <v>24</v>
-      </c>
-      <c r="J9" t="s">
+      <c r="G9" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H9" s="3">
+        <v>1853</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J9" s="3" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10">
+      <c r="A10" s="3">
         <v>2</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E10" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="E10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10">
-        <v>7706</v>
-      </c>
-      <c r="I10" t="s">
-        <v>24</v>
-      </c>
-      <c r="J10" t="s">
+      <c r="G10" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H10" s="3">
+        <v>2172</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J10" s="3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11">
+      <c r="A11" s="3">
         <v>3</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E11" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="E11" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H11">
-        <v>1011</v>
-      </c>
-      <c r="I11" t="s">
-        <v>24</v>
-      </c>
-      <c r="J11" t="s">
+      <c r="F11" s="3" t="s">
         <v>33</v>
       </c>
+      <c r="G11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11" s="3">
+        <v>727</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12">
+      <c r="A12" s="3">
         <v>4</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H12" s="3">
+        <v>833</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>5</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H13" s="3">
+        <v>821</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J13" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C12" t="s">
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>6</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D14" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E14" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H14" s="3">
+        <v>833</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>7</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F12" t="s">
+      <c r="C15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G12" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H12">
-        <v>2264</v>
-      </c>
-      <c r="I12" t="s">
-        <v>24</v>
-      </c>
-      <c r="J12" t="s">
+      <c r="G15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H15" s="3">
+        <v>1858</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>8</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H16" s="3">
+        <v>1121</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>9</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H17" s="3">
+        <v>996</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>10</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H18" s="3">
+        <v>5582</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
+        <v>11</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H19" s="3">
+        <v>5289</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
+        <v>12</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H20" s="3">
+        <v>2520</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="3">
+        <v>13</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H21" s="3">
+        <v>2296</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J21" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>5</v>
-      </c>
-      <c r="B13" t="s">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
+        <v>14</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C22" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H22" s="3">
+        <v>1531</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
+        <v>15</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H23" s="3">
+        <v>1277</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="3">
+        <v>16</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H24" s="3">
+        <v>2627</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="3">
+        <v>17</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H25" s="3">
+        <v>1223</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="3">
+        <v>18</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H26" s="3">
+        <v>1179</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="3">
+        <v>19</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H27" s="3">
+        <v>3063</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="3">
         <v>20</v>
       </c>
-      <c r="D13" t="s">
+      <c r="B28" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E28" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H28" s="3">
+        <v>1557</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="3">
+        <v>21</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H29" s="3">
+        <v>1303</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="3">
+        <v>22</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H30" s="3">
+        <v>4441</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="3">
+        <v>23</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H31" s="3">
+        <v>1402</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="3">
+        <v>24</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F13" t="s">
-        <v>39</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H13">
-        <v>935</v>
-      </c>
-      <c r="I13" t="s">
-        <v>24</v>
-      </c>
-      <c r="J13" t="s">
+      <c r="C32" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H32" s="3">
+        <v>1599</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J32" s="3" t="s">
         <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="3">
+        <v>25</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H33" s="3">
+        <v>2706</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J33" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="3">
+        <v>26</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H34" s="3">
+        <v>2435</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="3">
+        <v>27</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H35" s="3">
+        <v>1628</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>